<commit_message>
Add in-app Help & Documents; refresh docs and release build
The User Guide, Setup & Administration Guide and Release Notes are now
embedded in the app (Help & Documents screen) with PDF and Word downloads,
so one shared link or file carries the complete application.
Help screen hides the scan toolbar (found by checking the live hosted app).
97 tests: 42 unit, 47 UI scenario, 8 Playwright E2E.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QfiqXwchet7ZW5QeCH3Hw6
</commit_message>
<xml_diff>
--- a/sample-exports/Root_inventory_fixture.xlsx
+++ b/sample-exports/Root_inventory_fixture.xlsx
@@ -52,7 +52,7 @@
     <t>Started</t>
   </si>
   <si>
-    <t>2026-10-24 17:44</t>
+    <t>2026-10-24 18:21</t>
   </si>
   <si>
     <t>Completed</t>
@@ -61,7 +61,7 @@
     <t>Duration</t>
   </si>
   <si>
-    <t>8 ms</t>
+    <t>6 ms</t>
   </si>
   <si>
     <t>Files</t>

</xml_diff>